<commit_message>
Clean repo, add gitignore, update template
</commit_message>
<xml_diff>
--- a/Master_Valuation_Template_Clean_And_Final.xlsx
+++ b/Master_Valuation_Template_Clean_And_Final.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\janus\Desktop\Chat GPT uploads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Janus\Desktop\valuation-export-api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9679F07A-6D3F-4BD8-8893-0F5153DCBD72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A514EB1-6F07-4820-89CD-DE02DEE67EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet5!$A$1:$K$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet5!$A$1:$K$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="32">
   <si>
     <t>MARKET VALUATION</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>Proposed Price Calculated per Square Meter</t>
-  </si>
-  <si>
-    <t>SUMMARY</t>
   </si>
   <si>
     <t>Taking the market analysis and the condition of the property in to account, 
@@ -142,13 +139,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="6">
+  <numFmts count="5">
+    <numFmt numFmtId="42" formatCode="_-&quot;R&quot;* #,##0_-;\-&quot;R&quot;* #,##0_-;_-&quot;R&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="165" formatCode="_-&quot;R&quot;* #,##0_-;\-&quot;R&quot;* #,##0_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-&quot;R&quot;* #,##0_-;\-&quot;R&quot;* #,##0_-;_-&quot;R&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="169" formatCode="&quot;R&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="_-&quot;R&quot;* #,##0.00_-;\-&quot;R&quot;* #,##0.00_-;_-&quot;R&quot;* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -235,7 +231,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -274,18 +270,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF3399"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -304,15 +294,6 @@
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -372,7 +353,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -403,11 +384,11 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="42" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -426,86 +407,70 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -857,7 +822,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:N42"/>
+  <dimension ref="B1:N37"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.81640625" customWidth="1"/>
@@ -865,67 +830,67 @@
     <col min="3" max="3" width="6.81640625" customWidth="1"/>
     <col min="4" max="4" width="24.81640625" customWidth="1"/>
     <col min="5" max="6" width="8.81640625" customWidth="1"/>
-    <col min="7" max="7" width="11.1796875" style="43" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.1796875" style="37" bestFit="1" customWidth="1"/>
     <col min="8" max="10" width="6.81640625" customWidth="1"/>
     <col min="11" max="11" width="15.81640625" style="9" customWidth="1"/>
     <col min="13" max="13" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="23.4" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B1" s="48" t="s">
+      <c r="B1" s="51" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="50"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="46"/>
     </row>
     <row r="2" spans="2:13" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="60" t="s">
+      <c r="B2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="59"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
+      <c r="K2" s="43"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49"/>
-      <c r="J4" s="49"/>
-      <c r="K4" s="50"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="45"/>
+      <c r="F4" s="45"/>
+      <c r="G4" s="45"/>
+      <c r="H4" s="45"/>
+      <c r="I4" s="45"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="46"/>
     </row>
     <row r="6" spans="2:13" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="54" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="50"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="45"/>
+      <c r="F6" s="45"/>
+      <c r="G6" s="45"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="46"/>
     </row>
     <row r="7" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
@@ -937,10 +902,10 @@
       <c r="D7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="44" t="s">
+      <c r="E7" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="44" t="s">
+      <c r="F7" s="38" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="4" t="s">
@@ -969,7 +934,7 @@
       <c r="H8" s="17"/>
       <c r="I8" s="17"/>
       <c r="J8" s="17"/>
-      <c r="K8" s="29"/>
+      <c r="K8" s="28"/>
       <c r="M8" s="14" t="str">
         <f>IF(AND(ISNUMBER(K8), ISNUMBER(E8), E8&lt;&gt;0), K8/E8, "")</f>
         <v/>
@@ -985,7 +950,7 @@
       <c r="H9" s="17"/>
       <c r="I9" s="17"/>
       <c r="J9" s="17"/>
-      <c r="K9" s="29"/>
+      <c r="K9" s="28"/>
       <c r="M9" s="14" t="str">
         <f>IF(AND(ISNUMBER(K9), ISNUMBER(E9), E9&lt;&gt;0), K9/E9, "")</f>
         <v/>
@@ -1001,7 +966,7 @@
       <c r="H10" s="17"/>
       <c r="I10" s="17"/>
       <c r="J10" s="17"/>
-      <c r="K10" s="29"/>
+      <c r="K10" s="28"/>
       <c r="M10" s="14" t="str">
         <f>IF(AND(ISNUMBER(K10), ISNUMBER(E10), E10&lt;&gt;0), K10/E10, "")</f>
         <v/>
@@ -1012,12 +977,12 @@
       <c r="E11" s="21"/>
       <c r="F11" s="21"/>
       <c r="G11" s="22"/>
-      <c r="H11" s="55" t="s">
+      <c r="H11" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="49"/>
-      <c r="J11" s="50"/>
-      <c r="K11" s="31" t="str">
+      <c r="I11" s="45"/>
+      <c r="J11" s="46"/>
+      <c r="K11" s="30" t="str">
         <f>IF(COUNT(K8:K10)=0,"",AVERAGE(K8:K10))</f>
         <v/>
       </c>
@@ -1033,18 +998,18 @@
       <c r="K12" s="16"/>
     </row>
     <row r="13" spans="2:13" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="51" t="s">
+      <c r="B13" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="49"/>
-      <c r="I13" s="49"/>
-      <c r="J13" s="49"/>
-      <c r="K13" s="50"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="45"/>
+      <c r="H13" s="45"/>
+      <c r="I13" s="45"/>
+      <c r="J13" s="45"/>
+      <c r="K13" s="46"/>
     </row>
     <row r="14" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
@@ -1056,10 +1021,10 @@
       <c r="D14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E14" s="44" t="s">
+      <c r="E14" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="F14" s="38" t="s">
         <v>8</v>
       </c>
       <c r="G14" s="4" t="s">
@@ -1088,7 +1053,7 @@
       <c r="H15" s="17"/>
       <c r="I15" s="17"/>
       <c r="J15" s="17"/>
-      <c r="K15" s="29"/>
+      <c r="K15" s="28"/>
       <c r="M15" s="14" t="str">
         <f>IF(AND(ISNUMBER(K15), ISNUMBER(E15), E15&lt;&gt;0), K15/E15, "")</f>
         <v/>
@@ -1104,7 +1069,7 @@
       <c r="H16" s="17"/>
       <c r="I16" s="17"/>
       <c r="J16" s="17"/>
-      <c r="K16" s="29"/>
+      <c r="K16" s="28"/>
       <c r="M16" s="14" t="str">
         <f>IF(AND(ISNUMBER(K16), ISNUMBER(E16), E16&lt;&gt;0), K16/E16, "")</f>
         <v/>
@@ -1120,7 +1085,7 @@
       <c r="H17" s="17"/>
       <c r="I17" s="17"/>
       <c r="J17" s="17"/>
-      <c r="K17" s="29"/>
+      <c r="K17" s="28"/>
       <c r="M17" s="14" t="str">
         <f>IF(AND(ISNUMBER(K17), ISNUMBER(E17), E17&lt;&gt;0), K17/E17, "")</f>
         <v/>
@@ -1131,12 +1096,12 @@
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
       <c r="G18" s="22"/>
-      <c r="H18" s="55" t="s">
+      <c r="H18" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="I18" s="49"/>
-      <c r="J18" s="50"/>
-      <c r="K18" s="30" t="str">
+      <c r="I18" s="45"/>
+      <c r="J18" s="46"/>
+      <c r="K18" s="29" t="str">
         <f>IF(COUNT(K15:K17)=0,"",AVERAGE(K15:K17))</f>
         <v/>
       </c>
@@ -1155,18 +1120,18 @@
       </c>
     </row>
     <row r="20" spans="2:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="52" t="s">
+      <c r="B20" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="49"/>
-      <c r="D20" s="49"/>
-      <c r="E20" s="49"/>
-      <c r="F20" s="49"/>
-      <c r="G20" s="49"/>
-      <c r="H20" s="49"/>
-      <c r="I20" s="49"/>
-      <c r="J20" s="49"/>
-      <c r="K20" s="50"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="45"/>
+      <c r="E20" s="45"/>
+      <c r="F20" s="45"/>
+      <c r="G20" s="45"/>
+      <c r="H20" s="45"/>
+      <c r="I20" s="45"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="46"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="9"/>
@@ -1179,13 +1144,13 @@
       </c>
       <c r="E21" s="12"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="42"/>
+      <c r="G21" s="36"/>
       <c r="H21" s="9"/>
       <c r="I21" s="9"/>
       <c r="J21" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="K21" s="32" t="str">
+      <c r="K21" s="31" t="str">
         <f>IFERROR(AVERAGE(K8:K10,K15:K17),"")</f>
         <v/>
       </c>
@@ -1198,7 +1163,7 @@
       <c r="D22" s="24"/>
       <c r="E22" s="12"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="42"/>
+      <c r="G22" s="36"/>
       <c r="H22" s="9"/>
       <c r="I22" s="9"/>
       <c r="J22" s="11" t="s">
@@ -1215,13 +1180,13 @@
       <c r="D23" s="11"/>
       <c r="E23" s="12"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="42"/>
+      <c r="G23" s="36"/>
       <c r="H23" s="9"/>
       <c r="I23" s="9"/>
       <c r="J23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="38" t="e">
+      <c r="K23" s="32" t="e">
         <f>K22*D22</f>
         <v>#VALUE!</v>
       </c>
@@ -1232,243 +1197,181 @@
       <c r="D24" s="9"/>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
-      <c r="G24" s="42"/>
+      <c r="G24" s="36"/>
       <c r="H24" s="9"/>
       <c r="I24" s="9"/>
       <c r="J24" s="9"/>
     </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="61" t="s">
+    <row r="26" spans="2:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="26"/>
+      <c r="C26" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="C25" s="49"/>
-      <c r="D25" s="49"/>
-      <c r="E25" s="49"/>
-      <c r="F25" s="49"/>
-      <c r="G25" s="49"/>
-      <c r="H25" s="49"/>
-      <c r="I25" s="49"/>
-      <c r="J25" s="49"/>
-      <c r="K25" s="50"/>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B26" s="1"/>
-      <c r="J26" s="35" t="str">
-        <f>B6</f>
-        <v>01 - SOLD PROPERTIES IN STREET, COMPLEX OR ESTATE</v>
-      </c>
-      <c r="K26" s="36" t="str">
-        <f>K11</f>
-        <v/>
-      </c>
+      <c r="D26" s="41"/>
+      <c r="E26" s="41"/>
+      <c r="F26" s="41"/>
+      <c r="G26" s="42"/>
+      <c r="H26" s="41"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="41"/>
+      <c r="K26" s="43"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B27" s="1"/>
-      <c r="J27" s="27" t="str">
-        <f>B13</f>
-        <v>02 - SOLD PROPERTIES IN SUBURB AND SURROUNDING AREA</v>
-      </c>
-      <c r="K27" s="33" t="str">
-        <f>K18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="2:14" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="1"/>
-      <c r="J28" s="37" t="str">
-        <f>B20</f>
-        <v>03 - SOLD LAND IN SUBURB AND SURROUNDING AREA - AVERAGE ERF PER SQUARE METER</v>
-      </c>
-      <c r="K28" s="45" t="e">
-        <f>K23</f>
+      <c r="D27" s="6"/>
+      <c r="E27" s="39">
+        <v>0.98</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" s="56" t="e">
+        <f>K23*E27</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="29" spans="2:14" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="K29" s="34" t="e">
-        <f>AVERAGEIFS(K26:K28, K26:K28, "&gt;=1")</f>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="D28" s="6"/>
+      <c r="E28" s="39">
+        <v>1.02</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="K28" s="56" t="e">
+        <f>K23*E28</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="I29" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J29" s="34">
+        <v>8.0500000000000002E-2</v>
+      </c>
+      <c r="K29" s="25" t="e">
+        <f>K28*J29</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="J30" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="K30" s="33" t="e">
+        <f>K28-K29</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="31" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="J31" s="8"/>
+      <c r="K31" s="33"/>
+    </row>
+    <row r="32" spans="2:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
+      <c r="F32" s="45"/>
+      <c r="G32" s="45"/>
+      <c r="H32" s="45"/>
+      <c r="I32" s="45"/>
+      <c r="J32" s="45"/>
+      <c r="K32" s="46"/>
+    </row>
+    <row r="33" spans="2:11" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F33" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="G33" s="46"/>
+      <c r="H33" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K33" s="15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="C34" s="3"/>
+      <c r="D34" s="23" t="e">
+        <f>K34/E34</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="31" spans="2:14" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="26"/>
-      <c r="C31" s="56" t="s">
-        <v>24</v>
-      </c>
-      <c r="D31" s="57"/>
-      <c r="E31" s="57"/>
-      <c r="F31" s="57"/>
-      <c r="G31" s="58"/>
-      <c r="H31" s="57"/>
-      <c r="I31" s="57"/>
-      <c r="J31" s="57"/>
-      <c r="K31" s="59"/>
-    </row>
-    <row r="32" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="D32" s="6"/>
-      <c r="E32" s="46">
-        <v>0.98</v>
-      </c>
-      <c r="J32" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="K32" s="47" t="e">
-        <f>K29*E32</f>
+      <c r="E34" s="17"/>
+      <c r="F34" s="49"/>
+      <c r="G34" s="46"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="28"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="23" t="e">
+        <f>K35/E35</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="D33" s="6"/>
-      <c r="E33" s="46">
-        <v>1.02</v>
-      </c>
-      <c r="J33" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="K33" s="47" t="e">
-        <f>K29*E33</f>
+      <c r="E35" s="17"/>
+      <c r="F35" s="49"/>
+      <c r="G35" s="46"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="28"/>
+    </row>
+    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="23" t="e">
+        <f>K36/E36</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="I34" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="J34" s="40">
-        <v>8.0500000000000002E-2</v>
-      </c>
-      <c r="K34" s="25" t="e">
-        <f>K33*J34</f>
+      <c r="E36" s="17"/>
+      <c r="F36" s="49"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="28"/>
+    </row>
+    <row r="37" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="C37" s="20"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="I37" s="45"/>
+      <c r="J37" s="46"/>
+      <c r="K37" s="35" t="e">
+        <f>AVERAGE(K34:K36)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="J35" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="K35" s="39" t="e">
-        <f>K33-K34</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="J36" s="8"/>
-      <c r="K36" s="39"/>
-    </row>
-    <row r="37" spans="2:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="64" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="49"/>
-      <c r="D37" s="49"/>
-      <c r="E37" s="49"/>
-      <c r="F37" s="49"/>
-      <c r="G37" s="49"/>
-      <c r="H37" s="49"/>
-      <c r="I37" s="49"/>
-      <c r="J37" s="49"/>
-      <c r="K37" s="50"/>
-    </row>
-    <row r="38" spans="2:11" ht="24.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E38" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F38" s="62" t="s">
-        <v>32</v>
-      </c>
-      <c r="G38" s="50"/>
-      <c r="H38" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="J38" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K38" s="15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="C39" s="3"/>
-      <c r="D39" s="23" t="e">
-        <f>K39/E39</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E39" s="17"/>
-      <c r="F39" s="63"/>
-      <c r="G39" s="50"/>
-      <c r="H39" s="17"/>
-      <c r="I39" s="17"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="29"/>
-    </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
-      <c r="D40" s="23" t="e">
-        <f>K40/E40</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E40" s="17"/>
-      <c r="F40" s="63"/>
-      <c r="G40" s="50"/>
-      <c r="H40" s="17"/>
-      <c r="I40" s="17"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="29"/>
-    </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="23" t="e">
-        <f>K41/E41</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="E41" s="17"/>
-      <c r="F41" s="63"/>
-      <c r="G41" s="50"/>
-      <c r="H41" s="17"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="17"/>
-      <c r="K41" s="29"/>
-    </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.35">
-      <c r="C42" s="20"/>
-      <c r="E42" s="21"/>
-      <c r="F42" s="21"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="55" t="s">
-        <v>14</v>
-      </c>
-      <c r="I42" s="49"/>
-      <c r="J42" s="50"/>
-      <c r="K42" s="41" t="e">
-        <f>AVERAGE(K39:K41)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="C31:K31"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="B25:K25"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="B37:K37"/>
+  <mergeCells count="15">
     <mergeCell ref="B1:K1"/>
     <mergeCell ref="B13:K13"/>
     <mergeCell ref="B20:K20"/>
@@ -1476,6 +1379,14 @@
     <mergeCell ref="C4:K4"/>
     <mergeCell ref="H11:J11"/>
     <mergeCell ref="H18:J18"/>
+    <mergeCell ref="C26:K26"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B32:K32"/>
   </mergeCells>
   <conditionalFormatting sqref="M8:M10">
     <cfRule type="expression" dxfId="3" priority="10">

</xml_diff>